<commit_message>
feat: implement MRP validation logic and expand backend engine and frontend services with accompanying test data.
</commit_message>
<xml_diff>
--- a/dummy_test_data/dummy.xlsx
+++ b/dummy_test_data/dummy.xlsx
@@ -1038,7 +1038,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="2">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>7</v>
@@ -1053,10 +1053,10 @@
         <v>10</v>
       </c>
       <c r="F2" s="1">
-        <v>15</v>
+        <v>17.1</v>
       </c>
       <c r="G2" s="1">
-        <v>1500</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>